<commit_message>
fix: address Computer Use QA findings
</commit_message>
<xml_diff>
--- a/docs/qa/Shogi_Computer_Use_Test_Tracker.xlsx
+++ b/docs/qa/Shogi_Computer_Use_Test_Tracker.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Rb861aba4fd6349cc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Cases" sheetId="2" r:id="R80bf6aff816a4117"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Execution" sheetId="3" r:id="Rdccd54d06d9f4954"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Issues" sheetId="4" r:id="R35abbdf4bc434240"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="5" r:id="R9be3ec276d564507"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R1277464df0754321"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Cases" sheetId="2" r:id="R7f0d84c351214cf5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Execution" sheetId="3" r:id="R3428c151cdb440c8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Issues" sheetId="4" r:id="R5ade9b1b7db240de"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="5" r:id="R2f680c285d894bfd"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -875,7 +875,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="ExecutionTable" displayName="ExecutionTable" ref="A4:O40" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="ExecutionTable" displayName="ExecutionTable" ref="A4:O47" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="15">
     <x:tableColumn id="1" name="Run ID"/>
     <x:tableColumn id="2" name="Environment"/>
@@ -1171,7 +1171,7 @@
         <x:v>対象リリース／コミット</x:v>
       </x:c>
       <x:c r="B5" s="15" t="str">
-        <x:v>GitHub Pages 公開版（2026-07-20確認）</x:v>
+        <x:v>GitHub Pages 公開版＋修正ブランチ再テスト（2026-07-20）</x:v>
       </x:c>
       <x:c r="C5" s="15"/>
       <x:c r="D5" s="22"/>
@@ -1240,43 +1240,43 @@
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="48" t="str">
-        <x:v>RUN-001</x:v>
+        <x:v>全実行ログ</x:v>
       </x:c>
       <x:c r="B11" s="55" t="n">
-        <x:f>COUNTA('Execution'!$E$5:$E$40)</x:f>
-        <x:v>36</x:v>
+        <x:f>COUNTA('Execution'!$E$5:$E$47)</x:f>
+        <x:v>43</x:v>
       </x:c>
       <x:c r="C11" s="55" t="n">
-        <x:f>COUNTIF('Execution'!$G$5:$G$40,"&lt;&gt;Not Run")-COUNTBLANK('Execution'!$G$5:$G$40)</x:f>
+        <x:f>COUNTIF('Execution'!$G$5:$G$47,"&lt;&gt;Not Run")-COUNTBLANK('Execution'!$G$5:$G$47)</x:f>
+        <x:v>33</x:v>
+      </x:c>
+      <x:c r="D11" s="55" t="n">
+        <x:f>COUNTIF('Execution'!$G$5:$G$47,"Pass")</x:f>
         <x:v>26</x:v>
       </x:c>
-      <x:c r="D11" s="55" t="n">
-        <x:f>COUNTIF('Execution'!$G$5:$G$40,"Pass")</x:f>
-        <x:v>19</x:v>
-      </x:c>
       <x:c r="E11" s="55" t="n">
-        <x:f>COUNTIF('Execution'!$G$5:$G$40,"Fail")</x:f>
+        <x:f>COUNTIF('Execution'!$G$5:$G$47,"Fail")</x:f>
         <x:v>6</x:v>
       </x:c>
       <x:c r="F11" s="55" t="n">
-        <x:f>COUNTIF('Execution'!$G$5:$G$40,"Blocked")</x:f>
+        <x:f>COUNTIF('Execution'!$G$5:$G$47,"Blocked")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="G11" s="55" t="n">
-        <x:f>COUNTIF('Execution'!$G$5:$G$40,"N/A")</x:f>
+        <x:f>COUNTIF('Execution'!$G$5:$G$47,"N/A")</x:f>
         <x:v>1</x:v>
       </x:c>
       <x:c r="H11" s="55" t="n">
-        <x:f>COUNTIF('Execution'!$G$5:$G$40,"Not Run")+COUNTBLANK('Execution'!$G$5:$G$40)</x:f>
+        <x:f>COUNTIF('Execution'!$G$5:$G$47,"Not Run")+COUNTBLANK('Execution'!$G$5:$G$47)</x:f>
         <x:v>10</x:v>
       </x:c>
       <x:c r="I11" s="57" t="n">
         <x:f>IFERROR(C11/B11,0)</x:f>
-        <x:v>0.7222222222222222</x:v>
+        <x:v>0.7674418604651163</x:v>
       </x:c>
       <x:c r="J11" s="56" t="n">
         <x:f>COUNTIFS('Issues'!$D$5:$D$54,"P0",'Issues'!$L$5:$L$54,"&lt;&gt;Fixed",'Issues'!$L$5:$L$54,"&lt;&gt;Won't Fix",'Issues'!$A$5:$A$54,"&lt;&gt;")+COUNTIFS('Issues'!$D$5:$D$54,"P1",'Issues'!$L$5:$L$54,"&lt;&gt;Fixed",'Issues'!$L$5:$L$54,"&lt;&gt;Won't Fix",'Issues'!$A$5:$A$54,"&lt;&gt;")</x:f>
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
@@ -1304,23 +1304,23 @@
         <x:v>ENV-01 Desktop</x:v>
       </x:c>
       <x:c r="B15" s="76" t="n">
-        <x:f>COUNTIF('Execution'!$B$5:$B$40,A15)</x:f>
-        <x:v>18</x:v>
+        <x:f>COUNTIF('Execution'!$B$5:$B$47,A15)</x:f>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="C15" s="76" t="n">
-        <x:f>COUNTIFS('Execution'!$B$5:$B$40,A15,'Execution'!$G$5:$G$40,"Pass")</x:f>
-        <x:v>9</x:v>
+        <x:f>COUNTIFS('Execution'!$B$5:$B$47,A15,'Execution'!$G$5:$G$47,"Pass")</x:f>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="D15" s="76" t="n">
-        <x:f>COUNTIFS('Execution'!$B$5:$B$40,A15,'Execution'!$G$5:$G$40,"Fail")</x:f>
+        <x:f>COUNTIFS('Execution'!$B$5:$B$47,A15,'Execution'!$G$5:$G$47,"Fail")</x:f>
         <x:v>3</x:v>
       </x:c>
       <x:c r="E15" s="76" t="n">
-        <x:f>COUNTIFS('Execution'!$B$5:$B$40,A15,'Execution'!$G$5:$G$40,"Blocked")</x:f>
+        <x:f>COUNTIFS('Execution'!$B$5:$B$47,A15,'Execution'!$G$5:$G$47,"Blocked")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="F15" s="77" t="n">
-        <x:f>COUNTIFS('Execution'!$B$5:$B$40,A15,'Execution'!$G$5:$G$40,"Not Run")+COUNTIFS('Execution'!$B$5:$B$40,A15,'Execution'!$G$5:$G$40,"")</x:f>
+        <x:f>COUNTIFS('Execution'!$B$5:$B$47,A15,'Execution'!$G$5:$G$47,"Not Run")+COUNTIFS('Execution'!$B$5:$B$47,A15,'Execution'!$G$5:$G$47,"")</x:f>
         <x:v>5</x:v>
       </x:c>
     </x:row>
@@ -1329,23 +1329,23 @@
         <x:v>ENV-02 Narrow</x:v>
       </x:c>
       <x:c r="B16" s="78" t="n">
-        <x:f>COUNTIF('Execution'!$B$5:$B$40,A16)</x:f>
-        <x:v>18</x:v>
+        <x:f>COUNTIF('Execution'!$B$5:$B$47,A16)</x:f>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="C16" s="78" t="n">
-        <x:f>COUNTIFS('Execution'!$B$5:$B$40,A16,'Execution'!$G$5:$G$40,"Pass")</x:f>
-        <x:v>10</x:v>
+        <x:f>COUNTIFS('Execution'!$B$5:$B$47,A16,'Execution'!$G$5:$G$47,"Pass")</x:f>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="D16" s="78" t="n">
-        <x:f>COUNTIFS('Execution'!$B$5:$B$40,A16,'Execution'!$G$5:$G$40,"Fail")</x:f>
+        <x:f>COUNTIFS('Execution'!$B$5:$B$47,A16,'Execution'!$G$5:$G$47,"Fail")</x:f>
         <x:v>3</x:v>
       </x:c>
       <x:c r="E16" s="78" t="n">
-        <x:f>COUNTIFS('Execution'!$B$5:$B$40,A16,'Execution'!$G$5:$G$40,"Blocked")</x:f>
+        <x:f>COUNTIFS('Execution'!$B$5:$B$47,A16,'Execution'!$G$5:$G$47,"Blocked")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="F16" s="79" t="n">
-        <x:f>COUNTIFS('Execution'!$B$5:$B$40,A16,'Execution'!$G$5:$G$40,"Not Run")+COUNTIFS('Execution'!$B$5:$B$40,A16,'Execution'!$G$5:$G$40,"")</x:f>
+        <x:f>COUNTIFS('Execution'!$B$5:$B$47,A16,'Execution'!$G$5:$G$47,"Not Run")+COUNTIFS('Execution'!$B$5:$B$47,A16,'Execution'!$G$5:$G$47,"")</x:f>
         <x:v>5</x:v>
       </x:c>
     </x:row>
@@ -2212,7 +2212,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd123702872394280"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2fb075234ccf424d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2259,7 +2259,7 @@
     </x:row>
     <x:row r="2" ht="22" customHeight="1">
       <x:c r="A2" s="9" t="str">
-        <x:v>RUN-001の実操作結果と、Desktop/Narrowの2環境×18ケースを記録しています。</x:v>
+        <x:v>RUN-001の初回実行とRUN-002のIssue再テストを、Desktop/Narrowの環境別に記録しています。</x:v>
       </x:c>
       <x:c r="B2" s="8"/>
       <x:c r="C2" s="8"/>
@@ -3727,46 +3727,347 @@
       </x:c>
     </x:row>
     <x:row r="40" ht="44" customHeight="1">
-      <x:c r="A40" s="110" t="str">
+      <x:c r="A40" s="108" t="str">
         <x:v>RUN-001</x:v>
       </x:c>
-      <x:c r="B40" s="111" t="str">
+      <x:c r="B40" s="109" t="str">
         <x:v>ENV-02 Narrow</x:v>
       </x:c>
-      <x:c r="C40" s="139" t="str"/>
-      <x:c r="D40" s="102" t="str"/>
-      <x:c r="E40" s="140" t="str">
+      <x:c r="C40" s="136" t="str"/>
+      <x:c r="D40" s="101" t="str"/>
+      <x:c r="E40" s="137" t="str">
         <x:v>CU-18</x:v>
       </x:c>
-      <x:c r="F40" s="140" t="str">
+      <x:c r="F40" s="137" t="str">
         <x:f>IFERROR(VLOOKUP(E40,'Test Cases'!$A$5:$C$22,3,FALSE),"")</x:f>
         <x:v>解析中止・連打・長棋譜</x:v>
       </x:c>
-      <x:c r="G40" s="102" t="str">
+      <x:c r="G40" s="101" t="str">
         <x:v>Not Run</x:v>
       </x:c>
-      <x:c r="H40" s="120" t="str">
+      <x:c r="H40" s="119" t="str">
         <x:f>IF(OR(G40="",G40="Not Run"),"☐","☑")</x:f>
         <x:v>☐</x:v>
       </x:c>
-      <x:c r="I40" s="141" t="str"/>
-      <x:c r="J40" s="123" t="str"/>
-      <x:c r="K40" s="123" t="str"/>
-      <x:c r="L40" s="123" t="str"/>
-      <x:c r="M40" s="123" t="str"/>
-      <x:c r="N40" s="123" t="str">
+      <x:c r="I40" s="138" t="str"/>
+      <x:c r="J40" s="122" t="str"/>
+      <x:c r="K40" s="122" t="str"/>
+      <x:c r="L40" s="122" t="str"/>
+      <x:c r="M40" s="122" t="str"/>
+      <x:c r="N40" s="122" t="str">
         <x:v>No</x:v>
       </x:c>
-      <x:c r="O40" s="126" t="str">
+      <x:c r="O40" s="125" t="str">
         <x:v>網羅不足としてRUN-001後に追加</x:v>
       </x:c>
+    </x:row>
+    <x:row r="41" ht="44" customHeight="1">
+      <x:c r="A41" s="108" t="str">
+        <x:v>RUN-002</x:v>
+      </x:c>
+      <x:c r="B41" s="109" t="str">
+        <x:v>ENV-01 Desktop</x:v>
+      </x:c>
+      <x:c r="C41" s="136" t="n">
+        <x:v>46223</x:v>
+      </x:c>
+      <x:c r="D41" s="101" t="str">
+        <x:v>Codex Computer Use</x:v>
+      </x:c>
+      <x:c r="E41" s="137" t="str">
+        <x:v>CU-04</x:v>
+      </x:c>
+      <x:c r="F41" s="137" t="str">
+        <x:f>IFERROR(VLOOKUP(E41,'Test Cases'!$A$5:$C$22,3,FALSE),"")</x:f>
+        <x:v>投了と新規対局</x:v>
+      </x:c>
+      <x:c r="G41" s="101" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="H41" s="119" t="str">
+        <x:f>IF(OR(G41="",G41="Not Run"),"☐","☑")</x:f>
+        <x:v>☑</x:v>
+      </x:c>
+      <x:c r="I41" s="138" t="str"/>
+      <x:c r="J41" s="122" t="str">
+        <x:v>docs/qa/evidence/RUN-002/CU-04-confirm-retest.jpeg</x:v>
+      </x:c>
+      <x:c r="K41" s="122" t="str">
+        <x:v>投了と新規対局の両方で影響説明付き確認を表示。安全側のキャンセルに初期フォーカスしEscape取消と確定後の状態更新を確認。</x:v>
+      </x:c>
+      <x:c r="L41" s="122" t="str">
+        <x:v>#7</x:v>
+      </x:c>
+      <x:c r="M41" s="122" t="str"/>
+      <x:c r="N41" s="122" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="O41" s="125" t="str"/>
+    </x:row>
+    <x:row r="42" ht="44" customHeight="1">
+      <x:c r="A42" s="108" t="str">
+        <x:v>RUN-002</x:v>
+      </x:c>
+      <x:c r="B42" s="109" t="str">
+        <x:v>ENV-01 Desktop</x:v>
+      </x:c>
+      <x:c r="C42" s="136" t="n">
+        <x:v>46223</x:v>
+      </x:c>
+      <x:c r="D42" s="101" t="str">
+        <x:v>Codex Computer Use</x:v>
+      </x:c>
+      <x:c r="E42" s="137" t="str">
+        <x:v>CU-06</x:v>
+      </x:c>
+      <x:c r="F42" s="137" t="str">
+        <x:f>IFERROR(VLOOKUP(E42,'Test Cases'!$A$5:$C$22,3,FALSE),"")</x:f>
+        <x:v>KIF読込（正常系）</x:v>
+      </x:c>
+      <x:c r="G42" s="101" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="H42" s="119" t="str">
+        <x:f>IF(OR(G42="",G42="Not Run"),"☐","☑")</x:f>
+        <x:v>☑</x:v>
+      </x:c>
+      <x:c r="I42" s="138" t="str"/>
+      <x:c r="J42" s="122" t="str">
+        <x:v>docs/qa/evidence/RUN-002/CU-06-kif-final-retest.jpeg</x:v>
+      </x:c>
+      <x:c r="K42" s="122" t="str">
+        <x:v>5手KIFの読込直後に5/5の最終局面と終局情報を表示。</x:v>
+      </x:c>
+      <x:c r="L42" s="122" t="str">
+        <x:v>#6</x:v>
+      </x:c>
+      <x:c r="M42" s="122" t="str"/>
+      <x:c r="N42" s="122" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="O42" s="125" t="str"/>
+    </x:row>
+    <x:row r="43" ht="44" customHeight="1">
+      <x:c r="A43" s="108" t="str">
+        <x:v>RUN-002</x:v>
+      </x:c>
+      <x:c r="B43" s="109" t="str">
+        <x:v>ENV-01 Desktop</x:v>
+      </x:c>
+      <x:c r="C43" s="136" t="n">
+        <x:v>46223</x:v>
+      </x:c>
+      <x:c r="D43" s="101" t="str">
+        <x:v>Codex Computer Use</x:v>
+      </x:c>
+      <x:c r="E43" s="137" t="str">
+        <x:v>CU-10</x:v>
+      </x:c>
+      <x:c r="F43" s="137" t="str">
+        <x:f>IFERROR(VLOOKUP(E43,'Test Cases'!$A$5:$C$22,3,FALSE),"")</x:f>
+        <x:v>URL共有</x:v>
+      </x:c>
+      <x:c r="G43" s="101" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="H43" s="119" t="str">
+        <x:f>IF(OR(G43="",G43="Not Run"),"☐","☑")</x:f>
+        <x:v>☑</x:v>
+      </x:c>
+      <x:c r="I43" s="138" t="str"/>
+      <x:c r="J43" s="122" t="str">
+        <x:v>docs/qa/evidence/RUN-002/CU-10-url-final-retest.jpeg</x:v>
+      </x:c>
+      <x:c r="K43" s="122" t="str">
+        <x:v>共有URLを直接開いた直後に同じ5手と5/5の最終局面を表示。新規対局後は古いmoves hashも消去。</x:v>
+      </x:c>
+      <x:c r="L43" s="122" t="str">
+        <x:v>#6</x:v>
+      </x:c>
+      <x:c r="M43" s="122" t="str"/>
+      <x:c r="N43" s="122" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="O43" s="125" t="str"/>
+    </x:row>
+    <x:row r="44" ht="44" customHeight="1">
+      <x:c r="A44" s="108" t="str">
+        <x:v>RUN-002</x:v>
+      </x:c>
+      <x:c r="B44" s="109" t="str">
+        <x:v>ENV-01 Desktop</x:v>
+      </x:c>
+      <x:c r="C44" s="136" t="n">
+        <x:v>46223</x:v>
+      </x:c>
+      <x:c r="D44" s="101" t="str">
+        <x:v>Codex Computer Use</x:v>
+      </x:c>
+      <x:c r="E44" s="137" t="str">
+        <x:v>CU-13</x:v>
+      </x:c>
+      <x:c r="F44" s="137" t="str">
+        <x:f>IFERROR(VLOOKUP(E44,'Test Cases'!$A$5:$C$22,3,FALSE),"")</x:f>
+        <x:v>キーボードフォーカスと読み上げ可能性</x:v>
+      </x:c>
+      <x:c r="G44" s="101" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="H44" s="119" t="str">
+        <x:f>IF(OR(G44="",G44="Not Run"),"☐","☑")</x:f>
+        <x:v>☑</x:v>
+      </x:c>
+      <x:c r="I44" s="138" t="str"/>
+      <x:c r="J44" s="122" t="str">
+        <x:v>docs/qa/evidence/RUN-002/CU-13-keyboard-retest.jpeg</x:v>
+      </x:c>
+      <x:c r="K44" s="122" t="str">
+        <x:v>Tabで盤へ到達し矢印キーとEnterだけで7七歩を7六へ着手。各マスは座標・所有者・駒種・選択状態を読み上げ可能。</x:v>
+      </x:c>
+      <x:c r="L44" s="122" t="str">
+        <x:v>#5</x:v>
+      </x:c>
+      <x:c r="M44" s="122" t="str"/>
+      <x:c r="N44" s="122" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="O44" s="125" t="str"/>
+    </x:row>
+    <x:row r="45" ht="44" customHeight="1">
+      <x:c r="A45" s="108" t="str">
+        <x:v>RUN-002</x:v>
+      </x:c>
+      <x:c r="B45" s="109" t="str">
+        <x:v>ENV-02 Narrow</x:v>
+      </x:c>
+      <x:c r="C45" s="136" t="n">
+        <x:v>46223</x:v>
+      </x:c>
+      <x:c r="D45" s="101" t="str">
+        <x:v>Codex Computer Use</x:v>
+      </x:c>
+      <x:c r="E45" s="137" t="str">
+        <x:v>CU-04</x:v>
+      </x:c>
+      <x:c r="F45" s="137" t="str">
+        <x:f>IFERROR(VLOOKUP(E45,'Test Cases'!$A$5:$C$22,3,FALSE),"")</x:f>
+        <x:v>投了と新規対局</x:v>
+      </x:c>
+      <x:c r="G45" s="101" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="H45" s="119" t="str">
+        <x:f>IF(OR(G45="",G45="Not Run"),"☐","☑")</x:f>
+        <x:v>☑</x:v>
+      </x:c>
+      <x:c r="I45" s="138" t="str"/>
+      <x:c r="J45" s="122" t="str">
+        <x:v>docs/qa/evidence/RUN-002/CU-04-confirm-narrow-retest.jpeg</x:v>
+      </x:c>
+      <x:c r="K45" s="122" t="str">
+        <x:v>Chrome DevTools Responsive 400px幅で確認文と両ボタンが収まりキャンセルへ初期フォーカス。</x:v>
+      </x:c>
+      <x:c r="L45" s="122" t="str">
+        <x:v>#7</x:v>
+      </x:c>
+      <x:c r="M45" s="122" t="str"/>
+      <x:c r="N45" s="122" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="O45" s="125" t="str"/>
+    </x:row>
+    <x:row r="46" ht="44" customHeight="1">
+      <x:c r="A46" s="108" t="str">
+        <x:v>RUN-002</x:v>
+      </x:c>
+      <x:c r="B46" s="109" t="str">
+        <x:v>ENV-02 Narrow</x:v>
+      </x:c>
+      <x:c r="C46" s="136" t="n">
+        <x:v>46223</x:v>
+      </x:c>
+      <x:c r="D46" s="101" t="str">
+        <x:v>Codex Computer Use</x:v>
+      </x:c>
+      <x:c r="E46" s="137" t="str">
+        <x:v>CU-06</x:v>
+      </x:c>
+      <x:c r="F46" s="137" t="str">
+        <x:f>IFERROR(VLOOKUP(E46,'Test Cases'!$A$5:$C$22,3,FALSE),"")</x:f>
+        <x:v>KIF読込（正常系）</x:v>
+      </x:c>
+      <x:c r="G46" s="101" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="H46" s="119" t="str">
+        <x:f>IF(OR(G46="",G46="Not Run"),"☐","☑")</x:f>
+        <x:v>☑</x:v>
+      </x:c>
+      <x:c r="I46" s="138" t="str"/>
+      <x:c r="J46" s="122" t="str">
+        <x:v>docs/qa/evidence/RUN-002/CU-06-kif-final-narrow-retest.jpeg</x:v>
+      </x:c>
+      <x:c r="K46" s="122" t="str">
+        <x:v>400px幅でも5手KIFの読込直後に5/5の最終局面と終局情報を表示。</x:v>
+      </x:c>
+      <x:c r="L46" s="122" t="str">
+        <x:v>#6</x:v>
+      </x:c>
+      <x:c r="M46" s="122" t="str"/>
+      <x:c r="N46" s="122" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="O46" s="125" t="str"/>
+    </x:row>
+    <x:row r="47" ht="44" customHeight="1">
+      <x:c r="A47" s="110" t="str">
+        <x:v>RUN-002</x:v>
+      </x:c>
+      <x:c r="B47" s="111" t="str">
+        <x:v>ENV-02 Narrow</x:v>
+      </x:c>
+      <x:c r="C47" s="139" t="n">
+        <x:v>46223</x:v>
+      </x:c>
+      <x:c r="D47" s="102" t="str">
+        <x:v>Codex Computer Use</x:v>
+      </x:c>
+      <x:c r="E47" s="140" t="str">
+        <x:v>CU-10</x:v>
+      </x:c>
+      <x:c r="F47" s="140" t="str">
+        <x:f>IFERROR(VLOOKUP(E47,'Test Cases'!$A$5:$C$22,3,FALSE),"")</x:f>
+        <x:v>URL共有</x:v>
+      </x:c>
+      <x:c r="G47" s="102" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="H47" s="120" t="str">
+        <x:f>IF(OR(G47="",G47="Not Run"),"☐","☑")</x:f>
+        <x:v>☑</x:v>
+      </x:c>
+      <x:c r="I47" s="141" t="str"/>
+      <x:c r="J47" s="123" t="str">
+        <x:v>docs/qa/evidence/RUN-002/CU-10-url-final-narrow-retest.jpeg</x:v>
+      </x:c>
+      <x:c r="K47" s="123" t="str">
+        <x:v>400px幅でも共有URLの初回表示が5/5の最終局面になり盤と操作部品の重なりなし。</x:v>
+      </x:c>
+      <x:c r="L47" s="123" t="str">
+        <x:v>#6</x:v>
+      </x:c>
+      <x:c r="M47" s="123" t="str"/>
+      <x:c r="N47" s="123" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="O47" s="126" t="str"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:O1"/>
     <x:mergeCell ref="A2:O2"/>
   </x:mergeCells>
-  <x:conditionalFormatting sqref="G5:G40">
+  <x:conditionalFormatting sqref="G5:G47">
     <x:cfRule type="containsText" dxfId="4" priority="1" operator="containsText" text="Not Run"/>
     <x:cfRule type="containsText" dxfId="5" priority="2" operator="containsText" text="Pass"/>
     <x:cfRule type="containsText" dxfId="6" priority="3" operator="containsText" text="Fail"/>
@@ -3774,19 +4075,19 @@
     <x:cfRule type="containsText" dxfId="8" priority="5" operator="containsText" text="N/A"/>
   </x:conditionalFormatting>
   <x:dataValidations count="3">
-    <x:dataValidation type="list" sqref="B5:B40">
+    <x:dataValidation type="list" sqref="B5:B47">
       <x:formula1>"ENV-01 Desktop,ENV-02 Narrow"</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="G5:G40">
+    <x:dataValidation type="list" sqref="G5:G47">
       <x:formula1>"Not Run,Pass,Fail,Blocked,N/A"</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="N5:N40">
+    <x:dataValidation type="list" sqref="N5:N47">
       <x:formula1>"No,Yes"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb68bcfb1ce6e46a0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb05ac0926fe7407b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3933,19 +4234,23 @@
         <x:v>ページ先頭からTab移動し盤上マスへの到達とアクセシビリティツリーを確認</x:v>
       </x:c>
       <x:c r="J5" s="121" t="str">
-        <x:v>docs/qa/evidence/RUN-001/CU-13-keyboard-focus-gap.png</x:v>
+        <x:v>docs/qa/evidence/RUN-002/CU-13-keyboard-retest.jpeg</x:v>
       </x:c>
       <x:c r="K5" s="121" t="str">
         <x:v>各マスへ座標・駒情報を含む名称とキーボード操作および可視フォーカスを追加</x:v>
       </x:c>
       <x:c r="L5" s="100" t="str">
-        <x:v>Open</x:v>
-      </x:c>
-      <x:c r="M5" s="100" t="str"/>
+        <x:v>Fixed</x:v>
+      </x:c>
+      <x:c r="M5" s="100" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
       <x:c r="N5" s="133" t="n">
         <x:v>46223</x:v>
       </x:c>
-      <x:c r="O5" s="133" t="str"/>
+      <x:c r="O5" s="133" t="n">
+        <x:v>46223</x:v>
+      </x:c>
       <x:c r="P5" s="103" t="str">
         <x:v>Now</x:v>
       </x:c>
@@ -3980,19 +4285,23 @@
         <x:v>5手KIFを読み込む。またはURL共有して新しいタブで開く</x:v>
       </x:c>
       <x:c r="J6" s="122" t="str">
-        <x:v>docs/qa/evidence/RUN-001/CU-06-valid-kif-loaded.png;docs/qa/evidence/RUN-001/CU-10-shared-url-restored.png</x:v>
+        <x:v>docs/qa/evidence/RUN-002/CU-06-kif-final-retest.jpeg;docs/qa/evidence/RUN-002/CU-10-url-final-retest.jpeg</x:v>
       </x:c>
       <x:c r="K6" s="122" t="str">
         <x:v>KIF読込とURL復元の完了時に表示位置を最終手へ同期</x:v>
       </x:c>
       <x:c r="L6" s="101" t="str">
-        <x:v>Open</x:v>
-      </x:c>
-      <x:c r="M6" s="101" t="str"/>
+        <x:v>Fixed</x:v>
+      </x:c>
+      <x:c r="M6" s="101" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
       <x:c r="N6" s="136" t="n">
         <x:v>46223</x:v>
       </x:c>
-      <x:c r="O6" s="136" t="str"/>
+      <x:c r="O6" s="136" t="n">
+        <x:v>46223</x:v>
+      </x:c>
       <x:c r="P6" s="104" t="str">
         <x:v>Next</x:v>
       </x:c>
@@ -4027,19 +4336,23 @@
         <x:v>1手以上指して投了を押す。再度棋譜を用意して新規対局を押す</x:v>
       </x:c>
       <x:c r="J7" s="122" t="str">
-        <x:v>docs/qa/evidence/RUN-001/CU-04-resign.png</x:v>
+        <x:v>docs/qa/evidence/RUN-002/CU-04-confirm-retest.jpeg;docs/qa/evidence/RUN-002/CU-04-confirm-narrow-retest.jpeg</x:v>
       </x:c>
       <x:c r="K7" s="122" t="str">
         <x:v>未保存棋譜または進行中対局がある場合に安全側へ初期フォーカスした確認を表示</x:v>
       </x:c>
       <x:c r="L7" s="101" t="str">
-        <x:v>Open</x:v>
-      </x:c>
-      <x:c r="M7" s="101" t="str"/>
+        <x:v>Fixed</x:v>
+      </x:c>
+      <x:c r="M7" s="101" t="str">
+        <x:v>Codex</x:v>
+      </x:c>
       <x:c r="N7" s="136" t="n">
         <x:v>46223</x:v>
       </x:c>
-      <x:c r="O7" s="136" t="str"/>
+      <x:c r="O7" s="136" t="n">
+        <x:v>46223</x:v>
+      </x:c>
       <x:c r="P7" s="104" t="str">
         <x:v>Next</x:v>
       </x:c>
@@ -5014,7 +5327,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R235db27457f946b8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R06ab4961a3b24d52"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>